<commit_message>
Actualizacion del excel Casos de Prueba con todos los casos de prueba del proyecto realizados y correctos.
</commit_message>
<xml_diff>
--- a/Documentación/Casos de Prueba VitalSY.xlsx
+++ b/Documentación/Casos de Prueba VitalSY.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07488097-4A8B-402D-A03A-CEE0F70626F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1B300A-9D44-44F4-B07B-DD566B4E5397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="176">
   <si>
     <t>CASOS DE PRUEBAS - [VitalSY]</t>
   </si>
@@ -272,12 +272,376 @@
   <si>
     <t>El archivo PDF fue generado exitosamente conteniendo las gráficas y registros del mes, con total legibilidad.</t>
   </si>
+  <si>
+    <t>ÁREA FUNCIONAL: Registro y Monitoreo de Glucosa (C.U 04, C.U 10, C.U 15)</t>
+  </si>
+  <si>
+    <t>CP-09</t>
+  </si>
+  <si>
+    <t>Registrar Lectura Manual de Glucosa (C.U 04)</t>
+  </si>
+  <si>
+    <t>El usuario está autenticado con JWT válido y se encuentra en la pantalla de registro de glucosa.</t>
+  </si>
+  <si>
+    <t>Glucosa: 145 mg/dL · Comentario: "Medición post-almuerzo"</t>
+  </si>
+  <si>
+    <t>El sistema almacena el registro en la tabla registros_glucemia vinculado al usuario autenticado con la fecha/hora actual. La nueva lectura aparece inmediatamente en el dashboard y la bitácora con el valor y la tendencia correcta.</t>
+  </si>
+  <si>
+    <t>La lectura se registró correctamente en la base de datos y se mostró de inmediato en el dashboard y la bitácora del paciente.</t>
+  </si>
+  <si>
+    <t>CP-10</t>
+  </si>
+  <si>
+    <t>Sincronización Automática con LibreLinkUp (C.U 15)</t>
+  </si>
+  <si>
+    <t>El paciente posee un sensor Freestyle Libre activo y cuenta de LibreLinkUp configurada. El backend está en ejecución.</t>
+  </si>
+  <si>
+    <t>Email LibreLinkUp: user@example.com · Password LibreLinkUp: *******</t>
+  </si>
+  <si>
+    <t>El sistema valida las credenciales contra la API de Abbott, activa la sincronización y el scheduler del backend importa automáticamente las lecturas del sensor cada 5 minutos en la tabla registros_glucemia. Las lecturas sincronizadas aparecen en el dashboard y la bitácora.</t>
+  </si>
+  <si>
+    <t>Las credenciales fueron validadas exitosamente. Las lecturas del sensor se sincronizaron automáticamente y aparecieron en la bitácora con sus timestamps originales.</t>
+  </si>
+  <si>
+    <t>CP-11</t>
+  </si>
+  <si>
+    <t>Visualizar Estadísticas de Tiempo en Rango – TIR (C.U 10)</t>
+  </si>
+  <si>
+    <t>El usuario tiene al menos 7 días de lecturas de glucosa registradas en la base de datos.</t>
+  </si>
+  <si>
+    <t>Periodo de consulta: Últimos 7 días</t>
+  </si>
+  <si>
+    <t>El sistema muestra un gráfico interactivo de línea con la evolución de glucosa y una barra tricolor con los porcentajes de tiempo en hipoglucemia (&lt;70 mg/dL), en rango (70-180 mg/dL) e hiperglucemia (&gt;180 mg/dL). Los datos son coherentes con las lecturas registradas.</t>
+  </si>
+  <si>
+    <t>Los gráficos se renderizaron correctamente con datos coherentes. La barra TIR mostró los porcentajes de distribución correspondientes al periodo seleccionado.</t>
+  </si>
+  <si>
+    <t>ÁREA FUNCIONAL: Inteligencia Artificial y Análisis Clínico (C.U 07, C.U 16, C.U 17, C.U 20)</t>
+  </si>
+  <si>
+    <t>CP-12</t>
+  </si>
+  <si>
+    <t>Generar Análisis Reactivo de Lectura con IA (C.U 07)</t>
+  </si>
+  <si>
+    <t>El backend tiene acceso a la API de Gemini. El paciente tiene datos basales completos en su perfil.</t>
+  </si>
+  <si>
+    <t>Glucosa registrada: 280 mg/dL (valor fuera de rango)</t>
+  </si>
+  <si>
+    <t>El backend estructura un prompt contextualizado con los datos basales del paciente y lo envía a Gemini. La respuesta generada contiene una recomendación clínica coherente y se asocia al registro de glucosa, siendo visible en la bitácora del paciente.</t>
+  </si>
+  <si>
+    <t>La IA generó un análisis clínico pertinente que se asoció correctamente al registro y se visualiza junto a la lectura en la bitácora.</t>
+  </si>
+  <si>
+    <t>CP-13</t>
+  </si>
+  <si>
+    <t>Chat Clínico Interactivo con IA (C.U 16)</t>
+  </si>
+  <si>
+    <t>El paciente tiene al menos 7 días de historial clínico registrado. El backend tiene acceso a la API de Gemini.</t>
+  </si>
+  <si>
+    <t>Consulta: "¿Cómo han sido mis niveles de glucosa esta semana?"</t>
+  </si>
+  <si>
+    <t>El backend extrae los últimos 7 días de bitácora, estructura un prompt contextualizado y consulta a Gemini. La respuesta es pertinente, personalizada y se renderiza correctamente en la interfaz de chat.</t>
+  </si>
+  <si>
+    <t>La IA respondió coherentemente haciendo referencia a los datos reales del paciente. La respuesta se renderizó correctamente en la interfaz de chat.</t>
+  </si>
+  <si>
+    <t>CP-14</t>
+  </si>
+  <si>
+    <t>Análisis Predictivo Causal con IA (C.U 17)</t>
+  </si>
+  <si>
+    <t>El paciente tiene al menos 7 días continuos de lecturas de glucemia registradas.</t>
+  </si>
+  <si>
+    <t>Periodo de análisis: Últimos 7 días</t>
+  </si>
+  <si>
+    <t>Gemini analiza los patrones causales de la bitácora, retorna una predicción de nivel de riesgo (Alto/Medio/Bajo) para las próximas 4 horas, identifica relaciones causa-efecto y ofrece recomendaciones preventivas. El resultado se persiste en alertas_predicciones.</t>
+  </si>
+  <si>
+    <t>El análisis identificó patrones causales correctamente, asignó un nivel de riesgo coherente y generó recomendaciones preventivas que se persistieron en la base de datos.</t>
+  </si>
+  <si>
+    <t>CP-15</t>
+  </si>
+  <si>
+    <t>Digitalización de Pauta Médica mediante OCR con IA (C.U 20)</t>
+  </si>
+  <si>
+    <t>Gemini procesa la imagen, extrae los rangos de glucemia y las dosis de insulina asociadas en formato JSON. La app presenta los datos para validación. Tras confirmación, la matriz de insulina se guarda como pauta activa del paciente en la base de datos.</t>
+  </si>
+  <si>
+    <t>La IA extrajo correctamente la matriz de dosis de la fotografía. Los datos fueron presentados, confirmados y guardados como pauta activa del paciente.</t>
+  </si>
+  <si>
+    <t>CP-16</t>
+  </si>
+  <si>
+    <t>Gestionar Alertas Proactivas por Valores Críticos (C.U 08)</t>
+  </si>
+  <si>
+    <t>El paciente tiene límites de seguridad configurados. Las notificaciones push están habilitadas en el dispositivo.</t>
+  </si>
+  <si>
+    <t>Glucosa registrada: 55 mg/dL (hipoglucemia severa)</t>
+  </si>
+  <si>
+    <t>La alerta de hipoglucemia se disparó correctamente con notificación push y modal emergente. La alerta fue registrada en la base de datos.</t>
+  </si>
+  <si>
+    <t>CP-17</t>
+  </si>
+  <si>
+    <t>Visualizar Bitácora Cronológica de Eventos (C.U 09)</t>
+  </si>
+  <si>
+    <t>El paciente tiene registros previos de glucemia, ingesta y dosis de insulina en la base de datos.</t>
+  </si>
+  <si>
+    <t>N/A (consulta de datos existentes)</t>
+  </si>
+  <si>
+    <t>Los eventos de glucosa, nutrición e insulina se muestran agrupados por día en orden descendente. Los acordeones interactivos permiten expandir/contraer cada grupo. El "pull-to-refresh" recarga los datos exitosamente. Los eventos se diferencian visualmente con íconos y colores apropiados.</t>
+  </si>
+  <si>
+    <t>La bitácora se renderizó correctamente con agrupación diaria, orden descendente e interacción fluida. La recarga actualizó los datos exitosamente.</t>
+  </si>
+  <si>
+    <t>CP-18</t>
+  </si>
+  <si>
+    <t>Configurar Recordatorios de Medición y Comidas (C.U 12)</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>El paciente está autenticado y tiene acceso a la sección de perfil/configuración.</t>
+  </si>
+  <si>
+    <t>Tipo: Comida · Hora: 13:00 · Repetición: Lunes a Viernes</t>
+  </si>
+  <si>
+    <t>El sistema almacena la preferencia de recordatorio en el backend. La configuración persiste correctamente tras cerrar y reabrir la aplicación.</t>
+  </si>
+  <si>
+    <t>La preferencia de recordatorio se almacenó correctamente y persistió tras reiniciar la aplicación. El scheduler de alertas temporizadas queda pendiente de implementación.</t>
+  </si>
+  <si>
+    <t>ÁREA FUNCIONAL: Recuperación de Acceso (C.U 14)</t>
+  </si>
+  <si>
+    <t>CP-19</t>
+  </si>
+  <si>
+    <t>Recuperación de Contraseña mediante Correo Electrónico (C.U 14)</t>
+  </si>
+  <si>
+    <t>El usuario tiene una cuenta registrada con un correo válido y accesible. El servicio de correo está operativo.</t>
+  </si>
+  <si>
+    <t>Email: seed@example.com</t>
+  </si>
+  <si>
+    <t>El sistema envía un correo con un token temporal de un solo uso. El formulario de cambio de contraseña permite establecer una nueva. Tras el cambio, el usuario puede autenticarse con la nueva contraseña. El token utilizado queda invalidado.</t>
+  </si>
+  <si>
+    <t>El correo se recibió exitosamente, el cambio de contraseña fue efectivo y la nueva contraseña se almacenó cifrada con BCrypt. El token fue invalidado tras su uso.</t>
+  </si>
+  <si>
+    <t>ÁREA FUNCIONAL: Administración del Sistema (C.U 18, C.U 19)</t>
+  </si>
+  <si>
+    <t>CP-20</t>
+  </si>
+  <si>
+    <t>Panel de Control y Gestión Administrativa de Usuarios (C.U 18)</t>
+  </si>
+  <si>
+    <t>El usuario ha iniciado sesión con un rol ADMIN válido. Existen al menos 2 pacientes registrados en el sistema.</t>
+  </si>
+  <si>
+    <t>El administrador puede ver la lista de usuarios, suspender una cuenta (atributo activo cambia a false) y habilitarla nuevamente. El paciente suspendido recibe un error al intentar autenticarse y puede volver a iniciar sesión tras ser habilitado.</t>
+  </si>
+  <si>
+    <t>La suspensión y habilitación de cuentas funcionó correctamente. El paciente suspendido no pudo autenticarse y tras ser habilitado accedió con normalidad.</t>
+  </si>
+  <si>
+    <t>CP-21</t>
+  </si>
+  <si>
+    <t>Monitoreo Clínico de Pacientes por Administrador (C.U 19)</t>
+  </si>
+  <si>
+    <t>El administrador está autenticado. El paciente seleccionado tiene lecturas de glucosa registradas.</t>
+  </si>
+  <si>
+    <t>El sistema muestra el perfil basal del paciente (nombre, peso, tipo de insulina) y renderiza un gráfico lineal con ng2-charts mostrando la evolución histórica de glucemias. El gráfico es interactivo y responsivo. Si no hay lecturas, muestra un mensaje de "sin datos disponibles".</t>
+  </si>
+  <si>
+    <t>El perfil del paciente y el gráfico de glucemias se cargaron correctamente. El gráfico fue interactivo y responsivo con datos coherentes.</t>
+  </si>
+  <si>
+    <t>1. Abrir la pantalla de registro de glucosa. 
+2. Ingresar el valor de glucemia (145 mg/dL). 
+3. Agregar un comentario opcional ("Medición post-almuerzo"). 
+4. Presionar 'Guardar lectura'. 
+5. Verificar en la bitácora y en la base de datos.</t>
+  </si>
+  <si>
+    <t>1. Ir a la sección de conectividad/sensores de la app. 
+2. Ingresar las credenciales de LibreLinkUp. 
+3. Presionar 'Conectar'. 
+4. Esperar 5 minutos para la primera ejecución del scheduler. 
+5. Verificar las nuevas lecturas importadas en la bitácora.</t>
+  </si>
+  <si>
+    <t>1. Ingresar al Dashboard principal. 
+2. Verificar que se muestre el gráfico lineal de evolución glucémica. 
+3. Verificar la barra tricolor de distribución TIR (hipoglucemia, en rango, hiperglucemia). 
+4. Validar que los porcentajes sumen 100%.</t>
+  </si>
+  <si>
+    <t>1. Registrar una lectura de glucosa de 280 mg/dL. 
+2. Verificar que el sistema envíe automáticamente los datos al motor de IA. 
+3. Esperar la respuesta del análisis clínico. 
+4. Verificar que la recomendación aparezca adjunta a la lectura en la bitácora.</t>
+  </si>
+  <si>
+    <t>1. Acceder a la sección del "Chat Clínico". 
+2. Escribir la consulta en el campo de texto. 
+3. Presionar 'Enviar'. 
+4. Verificar que la respuesta sea coherente con los datos reales del paciente.</t>
+  </si>
+  <si>
+    <t>1. Acceder a la sección de "Análisis Predictivo". 
+2. Solicitar el análisis de patrones. 
+3. Esperar la respuesta del motor predictivo. 
+4. Verificar la predicción de riesgo y las recomendaciones.</t>
+  </si>
+  <si>
+    <t>1. Acceder a la sección de "Bitácora" o "Historial". 
+2. Verificar que los eventos estén agrupados por día. 
+3. Verificar el orden cronológico descendente. 
+4. Expandir/contraer un grupo de eventos. 
+5. Ejecutar "pull-to-refresh".</t>
+  </si>
+  <si>
+    <t>1. Acceder a la configuración de recordatorios. 
+2. Activar el recordatorio de comidas. 
+3. Configurar la hora (13:00) y los días de repetición. 
+4. Guardar la configuración. 
+5. Cerrar y reabrir la app para verificar persistencia.</t>
+  </si>
+  <si>
+    <t>1. Ir a la pantalla de Login. 
+2. Seleccionar "Olvidé mi contraseña". 
+3. Ingresar el correo registrado. 
+4. Verificar la recepción del correo con el enlace de recuperación. 
+5. Acceder al enlace y cambiar la contraseña. 
+6. Iniciar sesión con la nueva contraseña.</t>
+  </si>
+  <si>
+    <t>1. Ingresar al Panel de Administración. 
+2. Verificar la lista de usuarios registrados. 
+3. Seleccionar un paciente. 
+4. Presionar "Suspender cuenta". 
+5. Verificar que el paciente no pueda iniciar sesión. 
+6. Presionar "Habilitar cuenta". 
+7. Verificar que el paciente pueda iniciar sesión nuevamente.</t>
+  </si>
+  <si>
+    <t>1. Desde el Panel de Administración, seleccionar un paciente. 
+2. Presionar "Ver detalle clínico". 
+3. Verificar la carga del perfil basal del paciente. 
+4. Verificar el gráfico interactivo de glucemias históricas.</t>
+  </si>
+  <si>
+    <t>1. Acceder a la sección de Calculadora / Pauta Médica. 
+2. Seleccionar "Digitalizar con foto". 
+3. Tomar fotografía de la receta médica. 
+4. Esperar el procesamiento OCR.                                         5. Validar los datos extraídos.
+6. Confirmar y guardar la pauta.</t>
+  </si>
+  <si>
+    <t>El sistema detecta el valor crítico, dispara una notificación push nativa de alta prioridad y despliega un modal de alerta con instrucciones ("Consume azucar rápido."). La alerta se registra en alertas_predicciones.</t>
+  </si>
+  <si>
+    <t>1. Registrar una lectura de glucosa de 55 mg/dL. y 25 g. de Carbohidratos 
+2. Verificar que se dispare una notificación push nativa. 
+3. Verificar que se abra un modal de alerta emergente con instrucciones. 
+4. Verificar el registro de la alerta en la base de datos.</t>
+  </si>
+  <si>
+    <t>Acción: Suspender cuenta del paciente Seed User</t>
+  </si>
+  <si>
+    <t>Paciente a consultar: Brayan Cárcamo</t>
+  </si>
+  <si>
+    <t>El paciente tiene acceso a los archivos del dispositivo. El backend tiene acceso al modelo multimodal de Gemini.</t>
+  </si>
+  <si>
+    <t>Imagen de una receta médica con tabla de dosis de insulina por rangos de glucosa.</t>
+  </si>
+  <si>
+    <t>CP-23</t>
+  </si>
+  <si>
+    <t>Validar Límites de Seguridad de Glucosa Inválidos (C.U 13 - Excepción)</t>
+  </si>
+  <si>
+    <t>El paciente está autenticado y se encuentra en la pantalla de Alertas de Glucosa del perfil.</t>
+  </si>
+  <si>
+    <t>Límite inferior (Hipoglicemia): 150 mg/dL · Límite superior (Hiperglicemia): 130 mg/dL (Rango inválido ya que el mínimo es mayor que el máximo).</t>
+  </si>
+  <si>
+    <t>El formulario activa el validador cruzado (rangoGlucosaValidator). Se despliega una alerta visual indicando "El mínimo debe ser menor al máximo". El botón "Guardar Alertas" se deshabilita para evitar el envío de datos inválidos y la base de datos no sufre cambios.</t>
+  </si>
+  <si>
+    <t>El sistema detectó el rango inválido mediante el validador reactivo, mostró la alerta visual de advertencia y bloqueó el botón de guardado.</t>
+  </si>
+  <si>
+    <t>ÁREA FUNCIONAL: Alertas, Bitácora y Recordatorios (C.U 08, C.U 09, C.U 12, CU13)</t>
+  </si>
+  <si>
+    <t>1. Acceder a Alertas de Glucosa en el perfil. 
+2. Intentar mover el slider de hipoglicemia (mínimo) a 150 mg/dL y el de hiperglicemia (máximo) a 130 mg/dL. 
+3. Observar la aparición de mensajes de advertencia. 
+4. Validar que el botón "Guardar Alertas" quede deshabilitado.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -301,6 +665,19 @@
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -322,7 +699,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -345,11 +722,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -366,11 +780,38 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -501,8 +942,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>9117093</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>3895723</xdr:rowOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>4080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -550,7 +991,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>19051</xdr:colOff>
+      <xdr:colOff>19052</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>1633613</xdr:rowOff>
     </xdr:to>
@@ -644,15 +1085,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>6400801</xdr:colOff>
+      <xdr:colOff>6853239</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>9524</xdr:rowOff>
+      <xdr:rowOff>80962</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>8216059</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>3937927</xdr:rowOff>
+      <xdr:colOff>8668497</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>56490</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -681,7 +1122,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14439901" y="16335374"/>
+          <a:off x="15235239" y="16392525"/>
           <a:ext cx="1815258" cy="3928403"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -800,7 +1241,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>258846</xdr:colOff>
+      <xdr:colOff>258847</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>3933825</xdr:rowOff>
     </xdr:to>
@@ -851,8 +1292,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>8210549</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>3971922</xdr:rowOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>5040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -900,7 +1341,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>305363</xdr:colOff>
+      <xdr:colOff>305364</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>3390900</xdr:rowOff>
     </xdr:to>
@@ -933,6 +1374,1026 @@
         <a:xfrm>
           <a:off x="16363951" y="28936950"/>
           <a:ext cx="2553262" cy="2924175"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>24411</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>11206</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>159112</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>585908</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D5B524D-861B-F3FC-C6FB-BE5CABD9D189}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19567470" y="35690735"/>
+          <a:ext cx="2311043" cy="3922059"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>8292355</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>11208</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>10505040</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>504264</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Imagen 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5FF68DAA-5525-6203-3993-3270245D69FC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16696767" y="41383326"/>
+          <a:ext cx="2212685" cy="3720350"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>11208</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>11205</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>102454</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>1557618</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Imagen 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{994076B7-5F23-345D-464A-C20DA6C955CC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19856826" y="54393352"/>
+          <a:ext cx="2267588" cy="3832413"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>504264</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>11206</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>64161</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>347382</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Imagen 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CFE83B3-9A1C-0D5A-E3E3-286D7B3EAE49}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22131617" y="56679353"/>
+          <a:ext cx="2473426" cy="4146176"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>22412</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>201705</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>617924</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>2474778</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Imagen 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2095B4C-ADA7-45B1-9E09-1B559AAF6514}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19868030" y="39119734"/>
+          <a:ext cx="2779057" cy="2987448"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>7776883</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>11205</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>11207</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>277611</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Imagen 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B2495730-3147-7F68-870C-5588D988D52E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16181295" y="32642734"/>
+          <a:ext cx="2745441" cy="2974227"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>11206</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>1826560</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>31217</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>386014</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Imagen 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43203157-0FAF-BB06-2089-D189528EE4C2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19856824" y="60590207"/>
+          <a:ext cx="2924735" cy="2940954"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>403412</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>1882589</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>554743</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>773206</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Imagen 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{73BCBC12-89D6-2CCD-9C6E-547F72D9DB87}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22759147" y="60646236"/>
+          <a:ext cx="3064862" cy="3272117"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>560294</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>120865</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>465000</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Imagen 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42DF2F0D-B655-3CE0-CF99-2C2D8D406688}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19845618" y="63895941"/>
+          <a:ext cx="8852648" cy="3133681"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>696368</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>188819</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>292955</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>923290</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Imagen 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8FD5652E-211F-C72C-3B2B-88DD145420E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="28495761" y="64006319"/>
+          <a:ext cx="2481301" cy="3591971"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>235322</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>560295</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>43</xdr:col>
+      <xdr:colOff>262530</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>782732</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Imagen 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C1905B84-6CA3-34E0-EEC3-068AE7713055}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="31331646" y="63895942"/>
+          <a:ext cx="11770973" cy="3451412"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>936491</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>25613</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>358398</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>104054</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Imagen 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2F6D758A-D653-BD6E-EA19-F58742490D80}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19864027" y="66700613"/>
+          <a:ext cx="5409050" cy="3316941"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>304800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1027" name="AutoShape 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4402C1CD-2476-6ED3-34EC-ECE24A94D24C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="19850100" y="44605575"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>304800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1028" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02F237E3-A0C7-205D-E54D-2E509300C803}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="19850100" y="44605575"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>392206</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>2319618</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>561895</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>747114</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DDFC3CA-81C4-3A35-8EAE-8F095224BB39}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19307735" y="43691736"/>
+          <a:ext cx="2554942" cy="3750290"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>224118</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>1994648</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>341625</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>437030</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="25" name="Imagen 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3775E2E9-173A-E3EA-679C-EAE73DEC50C5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21851471" y="46594060"/>
+          <a:ext cx="3031036" cy="3014382"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>324971</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>2162735</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>690467</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>33618</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="26" name="Imagen 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D687066A-78CA-3586-5D87-C7380AC333B3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19240500" y="48857647"/>
+          <a:ext cx="2750749" cy="3014383"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>336178</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>381002</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>246530</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>198669</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Imagen 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{286C2989-6C7D-F219-B758-8F04CABAF8F6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21963531" y="49552414"/>
+          <a:ext cx="9379322" cy="2484667"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>612324</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>1782534</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>337525</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>326571</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="Imagen 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{099DF5CF-C88A-91FA-7ED7-422301E8CAA6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19539860" y="55734855"/>
+          <a:ext cx="2106451" cy="3497037"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>108858</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>2000250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>129049</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>204108</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="30" name="Imagen 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{97D49648-0F45-BA63-D85B-5C3A32794756}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="24302358" y="55952571"/>
+          <a:ext cx="2183727" cy="3156858"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>8490857</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>1768928</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>80710</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>612320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="31" name="Imagen 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D0AEFD86-B53F-B981-ACE3-BF62611D92FF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16900071" y="60674249"/>
+          <a:ext cx="2108175" cy="3946071"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>-1</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>149678</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>13607</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>44766</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Imagen 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5039F719-2FAB-7971-F6C6-47193326CE00}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19866428" y="61340999"/>
+          <a:ext cx="2177143" cy="2711767"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>163285</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>232879</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="33" name="Imagen 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6EA0AC67-551B-55E2-4040-7A36352037A9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22029964" y="61354606"/>
+          <a:ext cx="2396415" cy="2748644"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1142,7 +2603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z13"/>
+  <dimension ref="A1:Z42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1151,25 +2612,24 @@
     <col min="4" max="4" width="19" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" customWidth="1"/>
     <col min="6" max="6" width="26.140625" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" customWidth="1"/>
     <col min="8" max="8" width="157.7109375" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="15.7109375" customWidth="1"/>
-    <col min="11" max="26" width="10.85546875" customWidth="1"/>
+    <col min="10" max="26" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -1220,17 +2680,17 @@
       </c>
     </row>
     <row r="3" spans="1:26" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
     </row>
     <row r="4" spans="1:26" ht="304.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -1349,17 +2809,17 @@
       </c>
     </row>
     <row r="8" spans="1:26" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
     </row>
     <row r="9" spans="1:26" ht="310.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
@@ -1449,17 +2909,17 @@
       </c>
     </row>
     <row r="12" spans="1:26" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
     </row>
     <row r="13" spans="1:26" ht="312.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
@@ -1477,7 +2937,7 @@
       <c r="E13" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="8" t="s">
         <v>69</v>
       </c>
       <c r="G13" s="5" t="s">
@@ -1490,12 +2950,511 @@
         <v>1</v>
       </c>
     </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+    </row>
+    <row r="15" spans="1:26" ht="213" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="263.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="195" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+    </row>
+    <row r="19" spans="1:9" ht="254.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="195" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="195" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="I22" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+    </row>
+    <row r="24" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+      <c r="A24" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="225" x14ac:dyDescent="0.25">
+      <c r="A25" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="I25" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+    </row>
+    <row r="28" spans="1:9" ht="180" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" s="16" customFormat="1" ht="206.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="I29" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="15"/>
+    </row>
+    <row r="31" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+      <c r="A31" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="I31" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="195" x14ac:dyDescent="0.25">
+      <c r="A32" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="I32" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="13"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="15"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="9"/>
+      <c r="B42" s="9"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="9"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="10">
+    <mergeCell ref="A33:I33"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A27:I27"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A8:I8"/>
     <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A14:I14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>